<commit_message>
complete processor logic implementation
</commit_message>
<xml_diff>
--- a/Microprogram.xlsx
+++ b/Microprogram.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30105"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30121"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Personal_Important\Facultate\Cursuri\ProiectAC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4F97DD43-72A8-4034-A22A-D24D4725BC76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A0FB3C08-142F-4E82-9196-9162EEE49651}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{49516754-8FBA-4519-B484-8BD7D17C2B2A}"/>
   </bookViews>
@@ -501,7 +501,7 @@
     <t>FOS_AD:</t>
   </si>
   <si>
-    <t>FOD_AD_B1: 0010101</t>
+    <t>FOD_AD_B1: 0010100</t>
   </si>
   <si>
     <t>FOS_AI:</t>
@@ -2062,7 +2062,7 @@
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15.6"/>
   <cols>
     <col min="1" max="1" width="14.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.28515625" style="3" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="10.140625" style="3" customWidth="1"/>
     <col min="3" max="3" width="15" style="3" customWidth="1"/>
     <col min="4" max="4" width="20.140625" style="3" customWidth="1"/>
     <col min="5" max="5" width="16.85546875" style="3" bestFit="1" customWidth="1"/>
@@ -3392,7 +3392,7 @@
         <v>000000000000000000000000110100111000</v>
       </c>
     </row>
-    <row r="16" spans="1:25" s="9" customFormat="1">
+    <row r="16" spans="1:25" s="9" customFormat="1" ht="15.75">
       <c r="A16" s="4" t="s">
         <v>148</v>
       </c>
@@ -3405,7 +3405,7 @@
       </c>
       <c r="D16" s="21" t="str">
         <f t="shared" si="0"/>
-        <v>0x000000D5A</v>
+        <v>0x000000E5A</v>
       </c>
       <c r="E16" s="16" t="s">
         <v>22</v>
@@ -3429,7 +3429,7 @@
         <v>33</v>
       </c>
       <c r="L16" s="17" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="M16" s="4" t="s">
         <v>26</v>
@@ -3467,7 +3467,7 @@
       </c>
       <c r="V16" s="9" t="str">
         <f t="shared" si="11"/>
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="W16" s="9" t="str">
         <f t="shared" si="12"/>
@@ -3479,7 +3479,7 @@
       </c>
       <c r="Y16" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>000000000000000000000000110101011010</v>
+        <v>000000000000000000000000111001011010</v>
       </c>
     </row>
     <row r="17" spans="1:25" s="9" customFormat="1">
@@ -3585,7 +3585,7 @@
       </c>
       <c r="D18" s="21" t="str">
         <f t="shared" si="0"/>
-        <v>0x201500B15</v>
+        <v>0x201500B14</v>
       </c>
       <c r="E18" s="16" t="s">
         <v>36</v>
@@ -3655,11 +3655,11 @@
       </c>
       <c r="X18" s="9" t="str">
         <f t="shared" si="13"/>
-        <v>0010101</v>
+        <v>0010100</v>
       </c>
       <c r="Y18" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>001000000001010100000000101100010101</v>
+        <v>001000000001010100000000101100010100</v>
       </c>
     </row>
     <row r="19" spans="1:25" s="9" customFormat="1">
@@ -4112,7 +4112,7 @@
         <v>000000000000000000000000100000000010</v>
       </c>
     </row>
-    <row r="24" spans="1:25" s="9" customFormat="1">
+    <row r="24" spans="1:25" s="9" customFormat="1" ht="15.75">
       <c r="A24" s="4" t="s">
         <v>161</v>
       </c>

</xml_diff>